<commit_message>
Feat: paso 2 con 5 ángulos, plantilla pre-diligenciada sin duplicados y UUID en keys S3
- Paso 2 reestructurado: 5 preguntas (una por ángulo de exploración) en lugar de una sola
- Interpolación {{paso_N}} ahora etiqueta cada respuesta con [Pregunta N: <enunciado>] cuando el paso tiene varias preguntas
- Prompt de mapa_de_oportunidades: nueva sección que explica los 5 ángulos a la IA y reglas para conservar diversidad de retos
- Plantilla xlsx: eliminadas 4 columnas duplicadas (cols 16-19 que repetían los títulos de 11-14)
- Bloque A del prompt reducido a 14 columnas — Hipótesis de impacto esperado queda vacía en el prefill para que el equipo la diligencie
- S3Service.generateKey ahora produce <prefix>/<nombre-original-slug>-<UUID><ext> para legibilidad + unicidad garantizada
- Removido npm run reset-data del vercel-build — los datos se conservan entre deploys

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/plantilla-priorizacion-mapa-oportunidades.xlsx
+++ b/apps/web/public/templates/plantilla-priorizacion-mapa-oportunidades.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="McZmAKy2RO4es6SormcAleubExrPozinBxm3QZC+WWQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="QkQJheViAf7BD0R8vYO5LlmyLtM4PLMzTE4Ri8IpVws="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
   <si>
     <t>Área</t>
   </si>
@@ -88,13 +88,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Problema o necesidad que motivó esta idea</t>
-  </si>
-  <si>
     <t>1-3</t>
-  </si>
-  <si>
-    <t>1-4</t>
   </si>
   <si>
     <t>CRITERIOS DE PRIORIZACIÓN DE OPORTUNIDADES DE IA</t>
@@ -280,7 +274,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -292,12 +285,10 @@
       <i/>
       <color rgb="FF444444"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <color rgb="FF444444"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -370,7 +361,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border/>
     <border>
       <left/>
@@ -384,11 +375,6 @@
       <bottom/>
     </border>
     <border>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <right/>
       <top/>
       <bottom/>
     </border>
@@ -424,14 +410,11 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -446,9 +429,6 @@
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -458,9 +438,6 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -468,14 +445,13 @@
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -705,7 +681,7 @@
     <col customWidth="1" min="11" max="11" width="15.0"/>
     <col customWidth="1" min="12" max="12" width="13.29"/>
     <col customWidth="1" min="13" max="13" width="8.0"/>
-    <col customWidth="1" min="14" max="28" width="8.71"/>
+    <col customWidth="1" min="14" max="24" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="56.25" customHeight="1">
@@ -754,104 +730,86 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="T1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="V1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="Z1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="W2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="X2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="Y2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z2" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA2" s="6"/>
+      <c r="Q2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W2" s="5"/>
     </row>
     <row r="9">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="12"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="9"/>
     </row>
     <row r="20" ht="15.75" customHeight="1"/>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1858,173 +1816,173 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="15"/>
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="D2" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="E2" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="F2" s="12" t="s">
         <v>30</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="D3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="E3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="F3" s="14" t="s">
         <v>36</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="D4" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="E4" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="F4" s="14" t="s">
         <v>42</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="D5" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="E5" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="F5" s="14" t="s">
         <v>48</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="D6" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="E6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="F6" s="14" t="s">
         <v>54</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="D7" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="E7" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="F7" s="14" t="s">
         <v>60</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="D8" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="E8" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="F8" s="14" t="s">
         <v>66</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="E9" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="F9" s="14" t="s">
         <v>72</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
chore(templates): eliminar columna hipótesis de impacto del mapa de oportunidades
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/plantilla-priorizacion-mapa-oportunidades.xlsx
+++ b/apps/web/public/templates/plantilla-priorizacion-mapa-oportunidades.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="QkQJheViAf7BD0R8vYO5LlmyLtM4PLMzTE4Ri8IpVws="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="tc3uVYaeMI1UD+a1qU73+VZ1wsRHwPeejWWcgiyUqXc="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>Área</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>Orientación sobre esfuerzo técnico</t>
-  </si>
-  <si>
-    <t>Hipótesis de impacto esperado</t>
   </si>
   <si>
     <t>Valor potencial</t>
@@ -263,7 +260,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -300,11 +297,6 @@
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
@@ -410,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -438,20 +430,17 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -681,7 +670,7 @@
     <col customWidth="1" min="11" max="11" width="15.0"/>
     <col customWidth="1" min="12" max="12" width="13.29"/>
     <col customWidth="1" min="13" max="13" width="8.0"/>
-    <col customWidth="1" min="14" max="24" width="8.71"/>
+    <col customWidth="1" min="14" max="23" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="56.25" customHeight="1">
@@ -745,14 +734,11 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" ht="18.0" customHeight="1">
@@ -770,29 +756,28 @@
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
+      <c r="O2" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="P2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="W2" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="V2" s="5"/>
     </row>
     <row r="9">
       <c r="A9" s="7"/>
@@ -809,7 +794,6 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
-      <c r="O9" s="9"/>
     </row>
     <row r="20" ht="15.75" customHeight="1"/>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1816,173 +1800,173 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="A1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="11" t="s">
         <v>29</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="E3" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="F3" s="13" t="s">
         <v>35</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="F4" s="13" t="s">
         <v>41</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="E5" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="F5" s="13" t="s">
         <v>47</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="C6" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="F6" s="13" t="s">
         <v>53</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="F7" s="13" t="s">
         <v>59</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="E8" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="F8" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="E9" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="F9" s="13" t="s">
         <v>71</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>